<commit_message>
Version 0.3.5, see CHANGELOG
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/src/pypelay/static_summary.xlsx
+++ b/src/pypelay/static_summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daveh\Github\J017-Sapura\pypelay\src\pypelay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F17214-C0D6-446E-A6B6-A6196629206A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F33F8D2-CC02-4C0F-A0C3-7D402535D11E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5265" yWindow="2190" windowWidth="16800" windowHeight="13170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="285" yWindow="810" windowWidth="29700" windowHeight="13530" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="83">
   <si>
     <t>Units</t>
   </si>
@@ -255,6 +255,33 @@
   </si>
   <si>
     <t>SNIF / SCF</t>
+  </si>
+  <si>
+    <t>Pipe forces and moments</t>
+  </si>
+  <si>
+    <t>Eff tension, overbend</t>
+  </si>
+  <si>
+    <t>Eff tension, stinger tip</t>
+  </si>
+  <si>
+    <t>Eff tension, sag bend</t>
+  </si>
+  <si>
+    <t>Bend moment, overbend</t>
+  </si>
+  <si>
+    <t>kNm</t>
+  </si>
+  <si>
+    <t>Bend moment, stinger tip</t>
+  </si>
+  <si>
+    <t>Bend moment, sag bend</t>
+  </si>
+  <si>
+    <t>Bend moment, weld repair</t>
   </si>
 </sst>
 </file>
@@ -302,7 +329,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -327,9 +354,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -664,13 +700,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH86"/>
+  <dimension ref="A1:AH95"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
     <col min="2" max="2" width="11.28515625" style="2" customWidth="1"/>
     <col min="3" max="14" width="10.28515625" style="4" customWidth="1"/>
-    <col min="15" max="22" width="10.28515625" customWidth="1"/>
+    <col min="15" max="22" width="10.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.25">
@@ -783,14 +819,14 @@
       <c r="L4" s="6"/>
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="11"/>
-      <c r="R4" s="11"/>
-      <c r="S4" s="11"/>
-      <c r="T4" s="11"/>
-      <c r="U4" s="11"/>
-      <c r="V4" s="11"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="10"/>
+      <c r="S4" s="10"/>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C5" s="6"/>
@@ -805,14 +841,14 @@
       <c r="L5" s="6"/>
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="11"/>
-      <c r="S5" s="11"/>
-      <c r="T5" s="11"/>
-      <c r="U5" s="11"/>
-      <c r="V5" s="11"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="10"/>
+      <c r="S5" s="10"/>
+      <c r="T5" s="10"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="10"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -831,14 +867,14 @@
       <c r="L6" s="6"/>
       <c r="M6" s="6"/>
       <c r="N6" s="6"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
-      <c r="R6" s="11"/>
-      <c r="S6" s="11"/>
-      <c r="T6" s="11"/>
-      <c r="U6" s="11"/>
-      <c r="V6" s="11"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="10"/>
+      <c r="Q6" s="10"/>
+      <c r="R6" s="10"/>
+      <c r="S6" s="10"/>
+      <c r="T6" s="10"/>
+      <c r="U6" s="10"/>
+      <c r="V6" s="10"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -859,14 +895,14 @@
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
       <c r="N7" s="6"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11"/>
-      <c r="R7" s="11"/>
-      <c r="S7" s="11"/>
-      <c r="T7" s="11"/>
-      <c r="U7" s="11"/>
-      <c r="V7" s="11"/>
+      <c r="O7" s="10"/>
+      <c r="P7" s="10"/>
+      <c r="Q7" s="10"/>
+      <c r="R7" s="10"/>
+      <c r="S7" s="10"/>
+      <c r="T7" s="10"/>
+      <c r="U7" s="10"/>
+      <c r="V7" s="10"/>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -887,14 +923,14 @@
       <c r="L8" s="6"/>
       <c r="M8" s="6"/>
       <c r="N8" s="6"/>
-      <c r="O8" s="11"/>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="11"/>
-      <c r="R8" s="11"/>
-      <c r="S8" s="11"/>
-      <c r="T8" s="11"/>
-      <c r="U8" s="11"/>
-      <c r="V8" s="11"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="10"/>
+      <c r="R8" s="10"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="10"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="10"/>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -1005,14 +1041,14 @@
       <c r="L14" s="5"/>
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
-      <c r="O14" s="9"/>
-      <c r="P14" s="9"/>
-      <c r="Q14" s="9"/>
-      <c r="R14" s="9"/>
-      <c r="S14" s="9"/>
-      <c r="T14" s="9"/>
-      <c r="U14" s="9"/>
-      <c r="V14" s="9"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="11"/>
+      <c r="Q14" s="11"/>
+      <c r="R14" s="11"/>
+      <c r="S14" s="11"/>
+      <c r="T14" s="11"/>
+      <c r="U14" s="11"/>
+      <c r="V14" s="11"/>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -1033,14 +1069,14 @@
       <c r="L15" s="5"/>
       <c r="M15" s="5"/>
       <c r="N15" s="5"/>
-      <c r="O15" s="9"/>
-      <c r="P15" s="9"/>
-      <c r="Q15" s="9"/>
-      <c r="R15" s="9"/>
-      <c r="S15" s="9"/>
-      <c r="T15" s="9"/>
-      <c r="U15" s="9"/>
-      <c r="V15" s="9"/>
+      <c r="O15" s="11"/>
+      <c r="P15" s="11"/>
+      <c r="Q15" s="11"/>
+      <c r="R15" s="11"/>
+      <c r="S15" s="11"/>
+      <c r="T15" s="11"/>
+      <c r="U15" s="11"/>
+      <c r="V15" s="11"/>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -1061,14 +1097,14 @@
       <c r="L16" s="5"/>
       <c r="M16" s="5"/>
       <c r="N16" s="5"/>
-      <c r="O16" s="9"/>
-      <c r="P16" s="9"/>
-      <c r="Q16" s="9"/>
-      <c r="R16" s="9"/>
-      <c r="S16" s="9"/>
-      <c r="T16" s="9"/>
-      <c r="U16" s="9"/>
-      <c r="V16" s="9"/>
+      <c r="O16" s="11"/>
+      <c r="P16" s="11"/>
+      <c r="Q16" s="11"/>
+      <c r="R16" s="11"/>
+      <c r="S16" s="11"/>
+      <c r="T16" s="11"/>
+      <c r="U16" s="11"/>
+      <c r="V16" s="11"/>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -1089,14 +1125,14 @@
       <c r="L17" s="5"/>
       <c r="M17" s="5"/>
       <c r="N17" s="5"/>
-      <c r="O17" s="9"/>
-      <c r="P17" s="9"/>
-      <c r="Q17" s="9"/>
-      <c r="R17" s="9"/>
-      <c r="S17" s="9"/>
-      <c r="T17" s="9"/>
-      <c r="U17" s="9"/>
-      <c r="V17" s="9"/>
+      <c r="O17" s="11"/>
+      <c r="P17" s="11"/>
+      <c r="Q17" s="11"/>
+      <c r="R17" s="11"/>
+      <c r="S17" s="11"/>
+      <c r="T17" s="11"/>
+      <c r="U17" s="11"/>
+      <c r="V17" s="11"/>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -1117,14 +1153,14 @@
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
       <c r="N18" s="5"/>
-      <c r="O18" s="9"/>
-      <c r="P18" s="9"/>
-      <c r="Q18" s="9"/>
-      <c r="R18" s="9"/>
-      <c r="S18" s="9"/>
-      <c r="T18" s="9"/>
-      <c r="U18" s="9"/>
-      <c r="V18" s="9"/>
+      <c r="O18" s="11"/>
+      <c r="P18" s="11"/>
+      <c r="Q18" s="11"/>
+      <c r="R18" s="11"/>
+      <c r="S18" s="11"/>
+      <c r="T18" s="11"/>
+      <c r="U18" s="11"/>
+      <c r="V18" s="11"/>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -1145,14 +1181,14 @@
       <c r="L19" s="6"/>
       <c r="M19" s="6"/>
       <c r="N19" s="6"/>
-      <c r="O19" s="11"/>
-      <c r="P19" s="11"/>
-      <c r="Q19" s="11"/>
-      <c r="R19" s="11"/>
-      <c r="S19" s="11"/>
-      <c r="T19" s="11"/>
-      <c r="U19" s="11"/>
-      <c r="V19" s="11"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="10"/>
+      <c r="S19" s="10"/>
+      <c r="T19" s="10"/>
+      <c r="U19" s="10"/>
+      <c r="V19" s="10"/>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -1173,14 +1209,14 @@
       <c r="L20" s="5"/>
       <c r="M20" s="5"/>
       <c r="N20" s="5"/>
-      <c r="O20" s="9"/>
-      <c r="P20" s="9"/>
-      <c r="Q20" s="9"/>
-      <c r="R20" s="9"/>
-      <c r="S20" s="9"/>
-      <c r="T20" s="9"/>
-      <c r="U20" s="9"/>
-      <c r="V20" s="9"/>
+      <c r="O20" s="11"/>
+      <c r="P20" s="11"/>
+      <c r="Q20" s="11"/>
+      <c r="R20" s="11"/>
+      <c r="S20" s="11"/>
+      <c r="T20" s="11"/>
+      <c r="U20" s="11"/>
+      <c r="V20" s="11"/>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -1201,14 +1237,14 @@
       <c r="L21" s="6"/>
       <c r="M21" s="6"/>
       <c r="N21" s="6"/>
-      <c r="O21" s="11"/>
-      <c r="P21" s="11"/>
-      <c r="Q21" s="11"/>
-      <c r="R21" s="11"/>
-      <c r="S21" s="11"/>
-      <c r="T21" s="11"/>
-      <c r="U21" s="11"/>
-      <c r="V21" s="11"/>
+      <c r="O21" s="10"/>
+      <c r="P21" s="10"/>
+      <c r="Q21" s="10"/>
+      <c r="R21" s="10"/>
+      <c r="S21" s="10"/>
+      <c r="T21" s="10"/>
+      <c r="U21" s="10"/>
+      <c r="V21" s="10"/>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -1229,14 +1265,14 @@
       <c r="L22" s="5"/>
       <c r="M22" s="5"/>
       <c r="N22" s="5"/>
-      <c r="O22" s="9"/>
-      <c r="P22" s="9"/>
-      <c r="Q22" s="9"/>
-      <c r="R22" s="9"/>
-      <c r="S22" s="9"/>
-      <c r="T22" s="9"/>
-      <c r="U22" s="9"/>
-      <c r="V22" s="9"/>
+      <c r="O22" s="11"/>
+      <c r="P22" s="11"/>
+      <c r="Q22" s="11"/>
+      <c r="R22" s="11"/>
+      <c r="S22" s="11"/>
+      <c r="T22" s="11"/>
+      <c r="U22" s="11"/>
+      <c r="V22" s="11"/>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
@@ -1257,14 +1293,14 @@
       <c r="L23" s="5"/>
       <c r="M23" s="5"/>
       <c r="N23" s="5"/>
-      <c r="O23" s="9"/>
-      <c r="P23" s="9"/>
-      <c r="Q23" s="9"/>
-      <c r="R23" s="9"/>
-      <c r="S23" s="9"/>
-      <c r="T23" s="9"/>
-      <c r="U23" s="9"/>
-      <c r="V23" s="9"/>
+      <c r="O23" s="11"/>
+      <c r="P23" s="11"/>
+      <c r="Q23" s="11"/>
+      <c r="R23" s="11"/>
+      <c r="S23" s="11"/>
+      <c r="T23" s="11"/>
+      <c r="U23" s="11"/>
+      <c r="V23" s="11"/>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
@@ -1291,14 +1327,14 @@
       <c r="L26" s="5"/>
       <c r="M26" s="5"/>
       <c r="N26" s="5"/>
-      <c r="O26" s="9"/>
-      <c r="P26" s="9"/>
-      <c r="Q26" s="9"/>
-      <c r="R26" s="9"/>
-      <c r="S26" s="9"/>
-      <c r="T26" s="9"/>
-      <c r="U26" s="9"/>
-      <c r="V26" s="9"/>
+      <c r="O26" s="11"/>
+      <c r="P26" s="11"/>
+      <c r="Q26" s="11"/>
+      <c r="R26" s="11"/>
+      <c r="S26" s="11"/>
+      <c r="T26" s="11"/>
+      <c r="U26" s="11"/>
+      <c r="V26" s="11"/>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
@@ -1319,14 +1355,14 @@
       <c r="L27" s="5"/>
       <c r="M27" s="5"/>
       <c r="N27" s="5"/>
-      <c r="O27" s="9"/>
-      <c r="P27" s="9"/>
-      <c r="Q27" s="9"/>
-      <c r="R27" s="9"/>
-      <c r="S27" s="9"/>
-      <c r="T27" s="9"/>
-      <c r="U27" s="9"/>
-      <c r="V27" s="9"/>
+      <c r="O27" s="11"/>
+      <c r="P27" s="11"/>
+      <c r="Q27" s="11"/>
+      <c r="R27" s="11"/>
+      <c r="S27" s="11"/>
+      <c r="T27" s="11"/>
+      <c r="U27" s="11"/>
+      <c r="V27" s="11"/>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
@@ -1347,14 +1383,14 @@
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
       <c r="N28" s="5"/>
-      <c r="O28" s="9"/>
-      <c r="P28" s="9"/>
-      <c r="Q28" s="9"/>
-      <c r="R28" s="9"/>
-      <c r="S28" s="9"/>
-      <c r="T28" s="9"/>
-      <c r="U28" s="9"/>
-      <c r="V28" s="9"/>
+      <c r="O28" s="11"/>
+      <c r="P28" s="11"/>
+      <c r="Q28" s="11"/>
+      <c r="R28" s="11"/>
+      <c r="S28" s="11"/>
+      <c r="T28" s="11"/>
+      <c r="U28" s="11"/>
+      <c r="V28" s="11"/>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -1375,14 +1411,14 @@
       <c r="L29" s="5"/>
       <c r="M29" s="5"/>
       <c r="N29" s="5"/>
-      <c r="O29" s="9"/>
-      <c r="P29" s="9"/>
-      <c r="Q29" s="9"/>
-      <c r="R29" s="9"/>
-      <c r="S29" s="9"/>
-      <c r="T29" s="9"/>
-      <c r="U29" s="9"/>
-      <c r="V29" s="9"/>
+      <c r="O29" s="11"/>
+      <c r="P29" s="11"/>
+      <c r="Q29" s="11"/>
+      <c r="R29" s="11"/>
+      <c r="S29" s="11"/>
+      <c r="T29" s="11"/>
+      <c r="U29" s="11"/>
+      <c r="V29" s="11"/>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
@@ -1403,14 +1439,14 @@
       <c r="L30" s="5"/>
       <c r="M30" s="5"/>
       <c r="N30" s="5"/>
-      <c r="O30" s="9"/>
-      <c r="P30" s="9"/>
-      <c r="Q30" s="9"/>
-      <c r="R30" s="9"/>
-      <c r="S30" s="9"/>
-      <c r="T30" s="9"/>
-      <c r="U30" s="9"/>
-      <c r="V30" s="9"/>
+      <c r="O30" s="11"/>
+      <c r="P30" s="11"/>
+      <c r="Q30" s="11"/>
+      <c r="R30" s="11"/>
+      <c r="S30" s="11"/>
+      <c r="T30" s="11"/>
+      <c r="U30" s="11"/>
+      <c r="V30" s="11"/>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
@@ -1431,14 +1467,14 @@
       <c r="L31" s="8"/>
       <c r="M31" s="8"/>
       <c r="N31" s="8"/>
-      <c r="O31" s="10"/>
-      <c r="P31" s="10"/>
-      <c r="Q31" s="10"/>
-      <c r="R31" s="10"/>
-      <c r="S31" s="10"/>
-      <c r="T31" s="10"/>
-      <c r="U31" s="10"/>
-      <c r="V31" s="10"/>
+      <c r="O31" s="12"/>
+      <c r="P31" s="12"/>
+      <c r="Q31" s="12"/>
+      <c r="R31" s="12"/>
+      <c r="S31" s="12"/>
+      <c r="T31" s="12"/>
+      <c r="U31" s="12"/>
+      <c r="V31" s="12"/>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -1459,14 +1495,14 @@
       <c r="L32" s="5"/>
       <c r="M32" s="5"/>
       <c r="N32" s="5"/>
-      <c r="O32" s="9"/>
-      <c r="P32" s="9"/>
-      <c r="Q32" s="9"/>
-      <c r="R32" s="9"/>
-      <c r="S32" s="9"/>
-      <c r="T32" s="9"/>
-      <c r="U32" s="9"/>
-      <c r="V32" s="9"/>
+      <c r="O32" s="11"/>
+      <c r="P32" s="11"/>
+      <c r="Q32" s="11"/>
+      <c r="R32" s="11"/>
+      <c r="S32" s="11"/>
+      <c r="T32" s="11"/>
+      <c r="U32" s="11"/>
+      <c r="V32" s="11"/>
       <c r="W32" s="9"/>
       <c r="X32" s="9"/>
       <c r="Y32" s="9"/>
@@ -1499,14 +1535,14 @@
       <c r="L33" s="5"/>
       <c r="M33" s="5"/>
       <c r="N33" s="5"/>
-      <c r="O33" s="9"/>
-      <c r="P33" s="9"/>
-      <c r="Q33" s="9"/>
-      <c r="R33" s="9"/>
-      <c r="S33" s="9"/>
-      <c r="T33" s="9"/>
-      <c r="U33" s="9"/>
-      <c r="V33" s="9"/>
+      <c r="O33" s="11"/>
+      <c r="P33" s="11"/>
+      <c r="Q33" s="11"/>
+      <c r="R33" s="11"/>
+      <c r="S33" s="11"/>
+      <c r="T33" s="11"/>
+      <c r="U33" s="11"/>
+      <c r="V33" s="11"/>
       <c r="W33" s="9"/>
       <c r="X33" s="9"/>
       <c r="Y33" s="9"/>
@@ -1539,14 +1575,14 @@
       <c r="L34" s="5"/>
       <c r="M34" s="5"/>
       <c r="N34" s="5"/>
-      <c r="O34" s="9"/>
-      <c r="P34" s="9"/>
-      <c r="Q34" s="9"/>
-      <c r="R34" s="9"/>
-      <c r="S34" s="9"/>
-      <c r="T34" s="9"/>
-      <c r="U34" s="9"/>
-      <c r="V34" s="9"/>
+      <c r="O34" s="11"/>
+      <c r="P34" s="11"/>
+      <c r="Q34" s="11"/>
+      <c r="R34" s="11"/>
+      <c r="S34" s="11"/>
+      <c r="T34" s="11"/>
+      <c r="U34" s="11"/>
+      <c r="V34" s="11"/>
       <c r="W34" s="9"/>
       <c r="X34" s="9"/>
       <c r="Y34" s="9"/>
@@ -1579,14 +1615,14 @@
       <c r="L35" s="5"/>
       <c r="M35" s="5"/>
       <c r="N35" s="5"/>
-      <c r="O35" s="9"/>
-      <c r="P35" s="9"/>
-      <c r="Q35" s="9"/>
-      <c r="R35" s="9"/>
-      <c r="S35" s="9"/>
-      <c r="T35" s="9"/>
-      <c r="U35" s="9"/>
-      <c r="V35" s="9"/>
+      <c r="O35" s="11"/>
+      <c r="P35" s="11"/>
+      <c r="Q35" s="11"/>
+      <c r="R35" s="11"/>
+      <c r="S35" s="11"/>
+      <c r="T35" s="11"/>
+      <c r="U35" s="11"/>
+      <c r="V35" s="11"/>
       <c r="W35" s="9"/>
       <c r="X35" s="9"/>
       <c r="Y35" s="9"/>
@@ -1602,99 +1638,99 @@
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="7"/>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
-      <c r="H38" s="7"/>
-      <c r="I38" s="7"/>
-      <c r="J38" s="7"/>
-      <c r="K38" s="7"/>
-      <c r="L38" s="7"/>
-      <c r="M38" s="7"/>
-      <c r="N38" s="7"/>
-      <c r="O38" s="12"/>
-      <c r="P38" s="12"/>
-      <c r="Q38" s="12"/>
-      <c r="R38" s="12"/>
-      <c r="S38" s="12"/>
-      <c r="T38" s="12"/>
-      <c r="U38" s="12"/>
-      <c r="V38" s="12"/>
+        <v>22</v>
+      </c>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5"/>
+      <c r="I38" s="5"/>
+      <c r="J38" s="5"/>
+      <c r="K38" s="5"/>
+      <c r="L38" s="5"/>
+      <c r="M38" s="5"/>
+      <c r="N38" s="5"/>
+      <c r="O38" s="5"/>
+      <c r="P38" s="5"/>
+      <c r="Q38" s="5"/>
+      <c r="R38" s="5"/>
+      <c r="S38" s="5"/>
+      <c r="T38" s="5"/>
+      <c r="U38" s="5"/>
+      <c r="V38" s="5"/>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C39" s="7"/>
-      <c r="D39" s="7"/>
-      <c r="E39" s="7"/>
-      <c r="F39" s="7"/>
-      <c r="G39" s="7"/>
-      <c r="H39" s="7"/>
-      <c r="I39" s="7"/>
-      <c r="J39" s="7"/>
-      <c r="K39" s="7"/>
-      <c r="L39" s="7"/>
-      <c r="M39" s="7"/>
-      <c r="N39" s="7"/>
-      <c r="O39" s="12"/>
-      <c r="P39" s="12"/>
-      <c r="Q39" s="12"/>
-      <c r="R39" s="12"/>
-      <c r="S39" s="12"/>
-      <c r="T39" s="12"/>
-      <c r="U39" s="12"/>
-      <c r="V39" s="12"/>
+        <v>22</v>
+      </c>
+      <c r="C39" s="5"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5"/>
+      <c r="H39" s="5"/>
+      <c r="I39" s="5"/>
+      <c r="J39" s="5"/>
+      <c r="K39" s="5"/>
+      <c r="L39" s="5"/>
+      <c r="M39" s="5"/>
+      <c r="N39" s="5"/>
+      <c r="O39" s="5"/>
+      <c r="P39" s="5"/>
+      <c r="Q39" s="5"/>
+      <c r="R39" s="5"/>
+      <c r="S39" s="5"/>
+      <c r="T39" s="5"/>
+      <c r="U39" s="5"/>
+      <c r="V39" s="5"/>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C40" s="7"/>
-      <c r="D40" s="7"/>
-      <c r="E40" s="7"/>
-      <c r="F40" s="7"/>
-      <c r="G40" s="7"/>
-      <c r="H40" s="7"/>
-      <c r="I40" s="7"/>
-      <c r="J40" s="7"/>
-      <c r="K40" s="7"/>
-      <c r="L40" s="7"/>
-      <c r="M40" s="7"/>
-      <c r="N40" s="7"/>
-      <c r="O40" s="12"/>
-      <c r="P40" s="12"/>
-      <c r="Q40" s="12"/>
-      <c r="R40" s="12"/>
-      <c r="S40" s="12"/>
-      <c r="T40" s="12"/>
-      <c r="U40" s="12"/>
-      <c r="V40" s="12"/>
+        <v>22</v>
+      </c>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+      <c r="I40" s="5"/>
+      <c r="J40" s="5"/>
+      <c r="K40" s="5"/>
+      <c r="L40" s="5"/>
+      <c r="M40" s="5"/>
+      <c r="N40" s="5"/>
+      <c r="O40" s="5"/>
+      <c r="P40" s="5"/>
+      <c r="Q40" s="5"/>
+      <c r="R40" s="5"/>
+      <c r="S40" s="5"/>
+      <c r="T40" s="5"/>
+      <c r="U40" s="5"/>
+      <c r="V40" s="5"/>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
@@ -1708,21 +1744,21 @@
       <c r="L41" s="5"/>
       <c r="M41" s="5"/>
       <c r="N41" s="5"/>
-      <c r="O41" s="5"/>
-      <c r="P41" s="5"/>
-      <c r="Q41" s="5"/>
-      <c r="R41" s="5"/>
-      <c r="S41" s="5"/>
-      <c r="T41" s="5"/>
-      <c r="U41" s="5"/>
-      <c r="V41" s="5"/>
+      <c r="O41" s="11"/>
+      <c r="P41" s="11"/>
+      <c r="Q41" s="11"/>
+      <c r="R41" s="11"/>
+      <c r="S41" s="11"/>
+      <c r="T41" s="11"/>
+      <c r="U41" s="11"/>
+      <c r="V41" s="11"/>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="5"/>
@@ -1736,21 +1772,21 @@
       <c r="L42" s="5"/>
       <c r="M42" s="5"/>
       <c r="N42" s="5"/>
-      <c r="O42" s="5"/>
-      <c r="P42" s="5"/>
-      <c r="Q42" s="5"/>
-      <c r="R42" s="5"/>
-      <c r="S42" s="5"/>
-      <c r="T42" s="5"/>
-      <c r="U42" s="5"/>
-      <c r="V42" s="5"/>
+      <c r="O42" s="11"/>
+      <c r="P42" s="11"/>
+      <c r="Q42" s="11"/>
+      <c r="R42" s="11"/>
+      <c r="S42" s="11"/>
+      <c r="T42" s="11"/>
+      <c r="U42" s="11"/>
+      <c r="V42" s="11"/>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5"/>
@@ -1764,73 +1800,73 @@
       <c r="L43" s="5"/>
       <c r="M43" s="5"/>
       <c r="N43" s="5"/>
-      <c r="O43" s="5"/>
-      <c r="P43" s="5"/>
-      <c r="Q43" s="5"/>
-      <c r="R43" s="5"/>
-      <c r="S43" s="5"/>
-      <c r="T43" s="5"/>
-      <c r="U43" s="5"/>
-      <c r="V43" s="5"/>
+      <c r="O43" s="11"/>
+      <c r="P43" s="11"/>
+      <c r="Q43" s="11"/>
+      <c r="R43" s="11"/>
+      <c r="S43" s="11"/>
+      <c r="T43" s="11"/>
+      <c r="U43" s="11"/>
+      <c r="V43" s="11"/>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C44" s="7"/>
-      <c r="D44" s="7"/>
-      <c r="E44" s="7"/>
-      <c r="F44" s="7"/>
-      <c r="G44" s="7"/>
-      <c r="H44" s="7"/>
-      <c r="I44" s="7"/>
-      <c r="J44" s="7"/>
-      <c r="K44" s="7"/>
-      <c r="L44" s="7"/>
-      <c r="M44" s="7"/>
-      <c r="N44" s="7"/>
-      <c r="O44" s="12"/>
-      <c r="P44" s="12"/>
-      <c r="Q44" s="12"/>
-      <c r="R44" s="12"/>
-      <c r="S44" s="12"/>
-      <c r="T44" s="12"/>
-      <c r="U44" s="12"/>
-      <c r="V44" s="12"/>
+        <v>79</v>
+      </c>
+      <c r="C44" s="5"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+      <c r="I44" s="5"/>
+      <c r="J44" s="5"/>
+      <c r="K44" s="5"/>
+      <c r="L44" s="5"/>
+      <c r="M44" s="5"/>
+      <c r="N44" s="5"/>
+      <c r="O44" s="11"/>
+      <c r="P44" s="11"/>
+      <c r="Q44" s="11"/>
+      <c r="R44" s="11"/>
+      <c r="S44" s="11"/>
+      <c r="T44" s="11"/>
+      <c r="U44" s="11"/>
+      <c r="V44" s="11"/>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="C45" s="7"/>
-      <c r="D45" s="7"/>
-      <c r="E45" s="7"/>
-      <c r="F45" s="7"/>
-      <c r="G45" s="7"/>
-      <c r="H45" s="7"/>
-      <c r="I45" s="7"/>
-      <c r="J45" s="7"/>
-      <c r="K45" s="7"/>
-      <c r="L45" s="7"/>
-      <c r="M45" s="7"/>
-      <c r="N45" s="7"/>
-      <c r="O45" s="12"/>
-      <c r="P45" s="12"/>
-      <c r="Q45" s="12"/>
-      <c r="R45" s="12"/>
-      <c r="S45" s="12"/>
-      <c r="T45" s="12"/>
-      <c r="U45" s="12"/>
-      <c r="V45" s="12"/>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+      <c r="I45" s="5"/>
+      <c r="J45" s="5"/>
+      <c r="K45" s="5"/>
+      <c r="L45" s="5"/>
+      <c r="M45" s="5"/>
+      <c r="N45" s="5"/>
+      <c r="O45" s="5"/>
+      <c r="P45" s="5"/>
+      <c r="Q45" s="5"/>
+      <c r="R45" s="5"/>
+      <c r="S45" s="5"/>
+      <c r="T45" s="5"/>
+      <c r="U45" s="5"/>
+      <c r="V45" s="5"/>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>2</v>
@@ -1847,18 +1883,18 @@
       <c r="L47" s="7"/>
       <c r="M47" s="7"/>
       <c r="N47" s="7"/>
-      <c r="O47" s="12"/>
-      <c r="P47" s="12"/>
-      <c r="Q47" s="12"/>
-      <c r="R47" s="12"/>
-      <c r="S47" s="12"/>
-      <c r="T47" s="12"/>
-      <c r="U47" s="12"/>
-      <c r="V47" s="12"/>
+      <c r="O47" s="13"/>
+      <c r="P47" s="13"/>
+      <c r="Q47" s="13"/>
+      <c r="R47" s="13"/>
+      <c r="S47" s="13"/>
+      <c r="T47" s="13"/>
+      <c r="U47" s="13"/>
+      <c r="V47" s="13"/>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>2</v>
@@ -1875,18 +1911,18 @@
       <c r="L48" s="7"/>
       <c r="M48" s="7"/>
       <c r="N48" s="7"/>
-      <c r="O48" s="12"/>
-      <c r="P48" s="12"/>
-      <c r="Q48" s="12"/>
-      <c r="R48" s="12"/>
-      <c r="S48" s="12"/>
-      <c r="T48" s="12"/>
-      <c r="U48" s="12"/>
-      <c r="V48" s="12"/>
+      <c r="O48" s="13"/>
+      <c r="P48" s="13"/>
+      <c r="Q48" s="13"/>
+      <c r="R48" s="13"/>
+      <c r="S48" s="13"/>
+      <c r="T48" s="13"/>
+      <c r="U48" s="13"/>
+      <c r="V48" s="13"/>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>2</v>
@@ -1903,102 +1939,102 @@
       <c r="L49" s="7"/>
       <c r="M49" s="7"/>
       <c r="N49" s="7"/>
-      <c r="O49" s="12"/>
-      <c r="P49" s="12"/>
-      <c r="Q49" s="12"/>
-      <c r="R49" s="12"/>
-      <c r="S49" s="12"/>
-      <c r="T49" s="12"/>
-      <c r="U49" s="12"/>
-      <c r="V49" s="12"/>
+      <c r="O49" s="13"/>
+      <c r="P49" s="13"/>
+      <c r="Q49" s="13"/>
+      <c r="R49" s="13"/>
+      <c r="S49" s="13"/>
+      <c r="T49" s="13"/>
+      <c r="U49" s="13"/>
+      <c r="V49" s="13"/>
     </row>
     <row r="50" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="7"/>
-      <c r="F50" s="7"/>
-      <c r="G50" s="7"/>
-      <c r="H50" s="7"/>
-      <c r="I50" s="7"/>
-      <c r="J50" s="7"/>
-      <c r="K50" s="7"/>
-      <c r="L50" s="7"/>
-      <c r="M50" s="7"/>
-      <c r="N50" s="7"/>
-      <c r="O50" s="12"/>
-      <c r="P50" s="12"/>
-      <c r="Q50" s="12"/>
-      <c r="R50" s="12"/>
-      <c r="S50" s="12"/>
-      <c r="T50" s="12"/>
-      <c r="U50" s="12"/>
-      <c r="V50" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="C50" s="5"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="5"/>
+      <c r="F50" s="5"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5"/>
+      <c r="I50" s="5"/>
+      <c r="J50" s="5"/>
+      <c r="K50" s="5"/>
+      <c r="L50" s="5"/>
+      <c r="M50" s="5"/>
+      <c r="N50" s="5"/>
+      <c r="O50" s="5"/>
+      <c r="P50" s="5"/>
+      <c r="Q50" s="5"/>
+      <c r="R50" s="5"/>
+      <c r="S50" s="5"/>
+      <c r="T50" s="5"/>
+      <c r="U50" s="5"/>
+      <c r="V50" s="5"/>
     </row>
     <row r="51" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C51" s="7"/>
-      <c r="D51" s="7"/>
-      <c r="E51" s="7"/>
-      <c r="F51" s="7"/>
-      <c r="G51" s="7"/>
-      <c r="H51" s="7"/>
-      <c r="I51" s="7"/>
-      <c r="J51" s="7"/>
-      <c r="K51" s="7"/>
-      <c r="L51" s="7"/>
-      <c r="M51" s="7"/>
-      <c r="N51" s="7"/>
-      <c r="O51" s="12"/>
-      <c r="P51" s="12"/>
-      <c r="Q51" s="12"/>
-      <c r="R51" s="12"/>
-      <c r="S51" s="12"/>
-      <c r="T51" s="12"/>
-      <c r="U51" s="12"/>
-      <c r="V51" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="K51" s="5"/>
+      <c r="L51" s="5"/>
+      <c r="M51" s="5"/>
+      <c r="N51" s="5"/>
+      <c r="O51" s="5"/>
+      <c r="P51" s="5"/>
+      <c r="Q51" s="5"/>
+      <c r="R51" s="5"/>
+      <c r="S51" s="5"/>
+      <c r="T51" s="5"/>
+      <c r="U51" s="5"/>
+      <c r="V51" s="5"/>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C52" s="7"/>
-      <c r="D52" s="7"/>
-      <c r="E52" s="7"/>
-      <c r="F52" s="7"/>
-      <c r="G52" s="7"/>
-      <c r="H52" s="7"/>
-      <c r="I52" s="7"/>
-      <c r="J52" s="7"/>
-      <c r="K52" s="7"/>
-      <c r="L52" s="7"/>
-      <c r="M52" s="7"/>
-      <c r="N52" s="7"/>
-      <c r="O52" s="12"/>
-      <c r="P52" s="12"/>
-      <c r="Q52" s="12"/>
-      <c r="R52" s="12"/>
-      <c r="S52" s="12"/>
-      <c r="T52" s="12"/>
-      <c r="U52" s="12"/>
-      <c r="V52" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="C52" s="5"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5"/>
+      <c r="I52" s="5"/>
+      <c r="J52" s="5"/>
+      <c r="K52" s="5"/>
+      <c r="L52" s="5"/>
+      <c r="M52" s="5"/>
+      <c r="N52" s="5"/>
+      <c r="O52" s="5"/>
+      <c r="P52" s="5"/>
+      <c r="Q52" s="5"/>
+      <c r="R52" s="5"/>
+      <c r="S52" s="5"/>
+      <c r="T52" s="5"/>
+      <c r="U52" s="5"/>
+      <c r="V52" s="5"/>
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>2</v>
@@ -2015,22 +2051,16 @@
       <c r="L53" s="7"/>
       <c r="M53" s="7"/>
       <c r="N53" s="7"/>
-      <c r="O53" s="12"/>
-      <c r="P53" s="12"/>
-      <c r="Q53" s="12"/>
-      <c r="R53" s="12"/>
-      <c r="S53" s="12"/>
-      <c r="T53" s="12"/>
-      <c r="U53" s="12"/>
-      <c r="V53" s="12"/>
+      <c r="O53" s="13"/>
+      <c r="P53" s="13"/>
+      <c r="Q53" s="13"/>
+      <c r="R53" s="13"/>
+      <c r="S53" s="13"/>
+      <c r="T53" s="13"/>
+      <c r="U53" s="13"/>
+      <c r="V53" s="13"/>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>68</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>2</v>
-      </c>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
       <c r="E54" s="7"/>
@@ -2043,297 +2073,274 @@
       <c r="L54" s="7"/>
       <c r="M54" s="7"/>
       <c r="N54" s="7"/>
-      <c r="O54" s="12"/>
-      <c r="P54" s="12"/>
-      <c r="Q54" s="12"/>
-      <c r="R54" s="12"/>
-      <c r="S54" s="12"/>
-      <c r="T54" s="12"/>
-      <c r="U54" s="12"/>
-      <c r="V54" s="12"/>
+      <c r="O54" s="13"/>
+      <c r="P54" s="13"/>
+      <c r="Q54" s="13"/>
+      <c r="R54" s="13"/>
+      <c r="S54" s="13"/>
+      <c r="T54" s="13"/>
+      <c r="U54" s="13"/>
+      <c r="V54" s="13"/>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="C55" s="7"/>
-      <c r="D55" s="7"/>
-      <c r="E55" s="7"/>
-      <c r="F55" s="7"/>
-      <c r="G55" s="7"/>
-      <c r="H55" s="7"/>
-      <c r="I55" s="7"/>
-      <c r="J55" s="7"/>
-      <c r="K55" s="7"/>
-      <c r="L55" s="7"/>
-      <c r="M55" s="7"/>
-      <c r="N55" s="7"/>
-      <c r="O55" s="12"/>
-      <c r="P55" s="12"/>
-      <c r="Q55" s="12"/>
-      <c r="R55" s="12"/>
-      <c r="S55" s="12"/>
-      <c r="T55" s="12"/>
-      <c r="U55" s="12"/>
-      <c r="V55" s="12"/>
+      <c r="A55" s="1" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>61</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C56" s="7"/>
+      <c r="D56" s="7"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="7"/>
+      <c r="G56" s="7"/>
+      <c r="H56" s="7"/>
+      <c r="I56" s="7"/>
+      <c r="J56" s="7"/>
+      <c r="K56" s="7"/>
+      <c r="L56" s="7"/>
+      <c r="M56" s="7"/>
+      <c r="N56" s="7"/>
+      <c r="O56" s="13"/>
+      <c r="P56" s="13"/>
+      <c r="Q56" s="13"/>
+      <c r="R56" s="13"/>
+      <c r="S56" s="13"/>
+      <c r="T56" s="13"/>
+      <c r="U56" s="13"/>
+      <c r="V56" s="13"/>
+    </row>
+    <row r="57" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>62</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C57" s="7"/>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="7"/>
+      <c r="J57" s="7"/>
+      <c r="K57" s="7"/>
+      <c r="L57" s="7"/>
+      <c r="M57" s="7"/>
+      <c r="N57" s="7"/>
+      <c r="O57" s="13"/>
+      <c r="P57" s="13"/>
+      <c r="Q57" s="13"/>
+      <c r="R57" s="13"/>
+      <c r="S57" s="13"/>
+      <c r="T57" s="13"/>
+      <c r="U57" s="13"/>
+      <c r="V57" s="13"/>
+    </row>
+    <row r="58" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>63</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C58" s="7"/>
+      <c r="D58" s="7"/>
+      <c r="E58" s="7"/>
+      <c r="F58" s="7"/>
+      <c r="G58" s="7"/>
+      <c r="H58" s="7"/>
+      <c r="I58" s="7"/>
+      <c r="J58" s="7"/>
+      <c r="K58" s="7"/>
+      <c r="L58" s="7"/>
+      <c r="M58" s="7"/>
+      <c r="N58" s="7"/>
+      <c r="O58" s="13"/>
+      <c r="P58" s="13"/>
+      <c r="Q58" s="13"/>
+      <c r="R58" s="13"/>
+      <c r="S58" s="13"/>
+      <c r="T58" s="13"/>
+      <c r="U58" s="13"/>
+      <c r="V58" s="13"/>
+    </row>
+    <row r="59" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>64</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C59" s="7"/>
+      <c r="D59" s="7"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="7"/>
+      <c r="G59" s="7"/>
+      <c r="H59" s="7"/>
+      <c r="I59" s="7"/>
+      <c r="J59" s="7"/>
+      <c r="K59" s="7"/>
+      <c r="L59" s="7"/>
+      <c r="M59" s="7"/>
+      <c r="N59" s="7"/>
+      <c r="O59" s="13"/>
+      <c r="P59" s="13"/>
+      <c r="Q59" s="13"/>
+      <c r="R59" s="13"/>
+      <c r="S59" s="13"/>
+      <c r="T59" s="13"/>
+      <c r="U59" s="13"/>
+      <c r="V59" s="13"/>
+    </row>
+    <row r="60" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>65</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C60" s="7"/>
+      <c r="D60" s="7"/>
+      <c r="E60" s="7"/>
+      <c r="F60" s="7"/>
+      <c r="G60" s="7"/>
+      <c r="H60" s="7"/>
+      <c r="I60" s="7"/>
+      <c r="J60" s="7"/>
+      <c r="K60" s="7"/>
+      <c r="L60" s="7"/>
+      <c r="M60" s="7"/>
+      <c r="N60" s="7"/>
+      <c r="O60" s="13"/>
+      <c r="P60" s="13"/>
+      <c r="Q60" s="13"/>
+      <c r="R60" s="13"/>
+      <c r="S60" s="13"/>
+      <c r="T60" s="13"/>
+      <c r="U60" s="13"/>
+      <c r="V60" s="13"/>
+    </row>
+    <row r="61" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>66</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C61" s="7"/>
+      <c r="D61" s="7"/>
+      <c r="E61" s="7"/>
+      <c r="F61" s="7"/>
+      <c r="G61" s="7"/>
+      <c r="H61" s="7"/>
+      <c r="I61" s="7"/>
+      <c r="J61" s="7"/>
+      <c r="K61" s="7"/>
+      <c r="L61" s="7"/>
+      <c r="M61" s="7"/>
+      <c r="N61" s="7"/>
+      <c r="O61" s="13"/>
+      <c r="P61" s="13"/>
+      <c r="Q61" s="13"/>
+      <c r="R61" s="13"/>
+      <c r="S61" s="13"/>
+      <c r="T61" s="13"/>
+      <c r="U61" s="13"/>
+      <c r="V61" s="13"/>
+    </row>
+    <row r="62" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>67</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C62" s="7"/>
+      <c r="D62" s="7"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="7"/>
+      <c r="G62" s="7"/>
+      <c r="H62" s="7"/>
+      <c r="I62" s="7"/>
+      <c r="J62" s="7"/>
+      <c r="K62" s="7"/>
+      <c r="L62" s="7"/>
+      <c r="M62" s="7"/>
+      <c r="N62" s="7"/>
+      <c r="O62" s="13"/>
+      <c r="P62" s="13"/>
+      <c r="Q62" s="13"/>
+      <c r="R62" s="13"/>
+      <c r="S62" s="13"/>
+      <c r="T62" s="13"/>
+      <c r="U62" s="13"/>
+      <c r="V62" s="13"/>
+    </row>
+    <row r="63" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>68</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C63" s="7"/>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="7"/>
+      <c r="G63" s="7"/>
+      <c r="H63" s="7"/>
+      <c r="I63" s="7"/>
+      <c r="J63" s="7"/>
+      <c r="K63" s="7"/>
+      <c r="L63" s="7"/>
+      <c r="M63" s="7"/>
+      <c r="N63" s="7"/>
+      <c r="O63" s="13"/>
+      <c r="P63" s="13"/>
+      <c r="Q63" s="13"/>
+      <c r="R63" s="13"/>
+      <c r="S63" s="13"/>
+      <c r="T63" s="13"/>
+      <c r="U63" s="13"/>
+      <c r="V63" s="13"/>
+    </row>
+    <row r="64" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="C64" s="7"/>
+      <c r="D64" s="7"/>
+      <c r="E64" s="7"/>
+      <c r="F64" s="7"/>
+      <c r="G64" s="7"/>
+      <c r="H64" s="7"/>
+      <c r="I64" s="7"/>
+      <c r="J64" s="7"/>
+      <c r="K64" s="7"/>
+      <c r="L64" s="7"/>
+      <c r="M64" s="7"/>
+      <c r="N64" s="7"/>
+      <c r="O64" s="13"/>
+      <c r="P64" s="13"/>
+      <c r="Q64" s="13"/>
+      <c r="R64" s="13"/>
+      <c r="S64" s="13"/>
+      <c r="T64" s="13"/>
+      <c r="U64" s="13"/>
+      <c r="V64" s="13"/>
+    </row>
+    <row r="65" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A57" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C57" s="5"/>
-      <c r="D57" s="5"/>
-      <c r="E57" s="5"/>
-      <c r="F57" s="5"/>
-      <c r="G57" s="5"/>
-      <c r="H57" s="5"/>
-      <c r="I57" s="5"/>
-      <c r="J57" s="5"/>
-      <c r="K57" s="5"/>
-      <c r="L57" s="5"/>
-      <c r="M57" s="5"/>
-      <c r="N57" s="5"/>
-      <c r="O57" s="9"/>
-      <c r="P57" s="9"/>
-      <c r="Q57" s="9"/>
-      <c r="R57" s="9"/>
-      <c r="S57" s="9"/>
-      <c r="T57" s="9"/>
-      <c r="U57" s="9"/>
-      <c r="V57" s="9"/>
-    </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A58" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C58" s="5"/>
-      <c r="D58" s="5"/>
-      <c r="E58" s="5"/>
-      <c r="F58" s="5"/>
-      <c r="G58" s="5"/>
-      <c r="H58" s="5"/>
-      <c r="I58" s="5"/>
-      <c r="J58" s="5"/>
-      <c r="K58" s="5"/>
-      <c r="L58" s="5"/>
-      <c r="M58" s="5"/>
-      <c r="N58" s="5"/>
-      <c r="O58" s="9"/>
-      <c r="P58" s="9"/>
-      <c r="Q58" s="9"/>
-      <c r="R58" s="9"/>
-      <c r="S58" s="9"/>
-      <c r="T58" s="9"/>
-      <c r="U58" s="9"/>
-      <c r="V58" s="9"/>
-    </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A59" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C59" s="5"/>
-      <c r="D59" s="5"/>
-      <c r="E59" s="5"/>
-      <c r="F59" s="5"/>
-      <c r="G59" s="5"/>
-      <c r="H59" s="5"/>
-      <c r="I59" s="5"/>
-      <c r="J59" s="5"/>
-      <c r="K59" s="5"/>
-      <c r="L59" s="5"/>
-      <c r="M59" s="5"/>
-      <c r="N59" s="5"/>
-      <c r="O59" s="9"/>
-      <c r="P59" s="9"/>
-      <c r="Q59" s="9"/>
-      <c r="R59" s="9"/>
-      <c r="S59" s="9"/>
-      <c r="T59" s="9"/>
-      <c r="U59" s="9"/>
-      <c r="V59" s="9"/>
-    </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A60" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C60" s="5"/>
-      <c r="D60" s="5"/>
-      <c r="E60" s="5"/>
-      <c r="F60" s="5"/>
-      <c r="G60" s="5"/>
-      <c r="H60" s="5"/>
-      <c r="I60" s="5"/>
-      <c r="J60" s="5"/>
-      <c r="K60" s="5"/>
-      <c r="L60" s="5"/>
-      <c r="M60" s="5"/>
-      <c r="N60" s="5"/>
-      <c r="O60" s="9"/>
-      <c r="P60" s="9"/>
-      <c r="Q60" s="9"/>
-      <c r="R60" s="9"/>
-      <c r="S60" s="9"/>
-      <c r="T60" s="9"/>
-      <c r="U60" s="9"/>
-      <c r="V60" s="9"/>
-    </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A61" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5"/>
-      <c r="E61" s="5"/>
-      <c r="F61" s="5"/>
-      <c r="G61" s="5"/>
-      <c r="H61" s="5"/>
-      <c r="I61" s="5"/>
-      <c r="J61" s="5"/>
-      <c r="K61" s="5"/>
-      <c r="L61" s="5"/>
-      <c r="M61" s="5"/>
-      <c r="N61" s="5"/>
-      <c r="O61" s="9"/>
-      <c r="P61" s="9"/>
-      <c r="Q61" s="9"/>
-      <c r="R61" s="9"/>
-      <c r="S61" s="9"/>
-      <c r="T61" s="9"/>
-      <c r="U61" s="9"/>
-      <c r="V61" s="9"/>
-    </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A62" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C62" s="5"/>
-      <c r="D62" s="5"/>
-      <c r="E62" s="5"/>
-      <c r="F62" s="5"/>
-      <c r="G62" s="5"/>
-      <c r="H62" s="5"/>
-      <c r="I62" s="5"/>
-      <c r="J62" s="5"/>
-      <c r="K62" s="5"/>
-      <c r="L62" s="5"/>
-      <c r="M62" s="5"/>
-      <c r="N62" s="5"/>
-      <c r="O62" s="9"/>
-      <c r="P62" s="9"/>
-      <c r="Q62" s="9"/>
-      <c r="R62" s="9"/>
-      <c r="S62" s="9"/>
-      <c r="T62" s="9"/>
-      <c r="U62" s="9"/>
-      <c r="V62" s="9"/>
-    </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A63" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
-      <c r="F63" s="5"/>
-      <c r="G63" s="5"/>
-      <c r="H63" s="5"/>
-      <c r="I63" s="5"/>
-      <c r="J63" s="5"/>
-      <c r="K63" s="5"/>
-      <c r="L63" s="5"/>
-      <c r="M63" s="5"/>
-      <c r="N63" s="5"/>
-      <c r="O63" s="9"/>
-      <c r="P63" s="9"/>
-      <c r="Q63" s="9"/>
-      <c r="R63" s="9"/>
-      <c r="S63" s="9"/>
-      <c r="T63" s="9"/>
-      <c r="U63" s="9"/>
-      <c r="V63" s="9"/>
-    </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A64" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C64" s="5"/>
-      <c r="D64" s="5"/>
-      <c r="E64" s="5"/>
-      <c r="F64" s="5"/>
-      <c r="G64" s="5"/>
-      <c r="H64" s="5"/>
-      <c r="I64" s="5"/>
-      <c r="J64" s="5"/>
-      <c r="K64" s="5"/>
-      <c r="L64" s="5"/>
-      <c r="M64" s="5"/>
-      <c r="N64" s="5"/>
-      <c r="O64" s="9"/>
-      <c r="P64" s="9"/>
-      <c r="Q64" s="9"/>
-      <c r="R64" s="9"/>
-      <c r="S64" s="9"/>
-      <c r="T64" s="9"/>
-      <c r="U64" s="9"/>
-      <c r="V64" s="9"/>
-    </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A65" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C65" s="5"/>
-      <c r="D65" s="5"/>
-      <c r="E65" s="5"/>
-      <c r="F65" s="5"/>
-      <c r="G65" s="5"/>
-      <c r="H65" s="5"/>
-      <c r="I65" s="5"/>
-      <c r="J65" s="5"/>
-      <c r="K65" s="5"/>
-      <c r="L65" s="5"/>
-      <c r="M65" s="5"/>
-      <c r="N65" s="5"/>
-      <c r="O65" s="9"/>
-      <c r="P65" s="9"/>
-      <c r="Q65" s="9"/>
-      <c r="R65" s="9"/>
-      <c r="S65" s="9"/>
-      <c r="T65" s="9"/>
-      <c r="U65" s="9"/>
-      <c r="V65" s="9"/>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>22</v>
@@ -2350,18 +2357,18 @@
       <c r="L66" s="5"/>
       <c r="M66" s="5"/>
       <c r="N66" s="5"/>
-      <c r="O66" s="9"/>
-      <c r="P66" s="9"/>
-      <c r="Q66" s="9"/>
-      <c r="R66" s="9"/>
-      <c r="S66" s="9"/>
-      <c r="T66" s="9"/>
-      <c r="U66" s="9"/>
-      <c r="V66" s="9"/>
+      <c r="O66" s="11"/>
+      <c r="P66" s="11"/>
+      <c r="Q66" s="11"/>
+      <c r="R66" s="11"/>
+      <c r="S66" s="11"/>
+      <c r="T66" s="11"/>
+      <c r="U66" s="11"/>
+      <c r="V66" s="11"/>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>22</v>
@@ -2378,18 +2385,18 @@
       <c r="L67" s="5"/>
       <c r="M67" s="5"/>
       <c r="N67" s="5"/>
-      <c r="O67" s="9"/>
-      <c r="P67" s="9"/>
-      <c r="Q67" s="9"/>
-      <c r="R67" s="9"/>
-      <c r="S67" s="9"/>
-      <c r="T67" s="9"/>
-      <c r="U67" s="9"/>
-      <c r="V67" s="9"/>
+      <c r="O67" s="11"/>
+      <c r="P67" s="11"/>
+      <c r="Q67" s="11"/>
+      <c r="R67" s="11"/>
+      <c r="S67" s="11"/>
+      <c r="T67" s="11"/>
+      <c r="U67" s="11"/>
+      <c r="V67" s="11"/>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>22</v>
@@ -2406,18 +2413,18 @@
       <c r="L68" s="5"/>
       <c r="M68" s="5"/>
       <c r="N68" s="5"/>
-      <c r="O68" s="9"/>
-      <c r="P68" s="9"/>
-      <c r="Q68" s="9"/>
-      <c r="R68" s="9"/>
-      <c r="S68" s="9"/>
-      <c r="T68" s="9"/>
-      <c r="U68" s="9"/>
-      <c r="V68" s="9"/>
+      <c r="O68" s="11"/>
+      <c r="P68" s="11"/>
+      <c r="Q68" s="11"/>
+      <c r="R68" s="11"/>
+      <c r="S68" s="11"/>
+      <c r="T68" s="11"/>
+      <c r="U68" s="11"/>
+      <c r="V68" s="11"/>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>22</v>
@@ -2434,18 +2441,18 @@
       <c r="L69" s="5"/>
       <c r="M69" s="5"/>
       <c r="N69" s="5"/>
-      <c r="O69" s="9"/>
-      <c r="P69" s="9"/>
-      <c r="Q69" s="9"/>
-      <c r="R69" s="9"/>
-      <c r="S69" s="9"/>
-      <c r="T69" s="9"/>
-      <c r="U69" s="9"/>
-      <c r="V69" s="9"/>
+      <c r="O69" s="11"/>
+      <c r="P69" s="11"/>
+      <c r="Q69" s="11"/>
+      <c r="R69" s="11"/>
+      <c r="S69" s="11"/>
+      <c r="T69" s="11"/>
+      <c r="U69" s="11"/>
+      <c r="V69" s="11"/>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>22</v>
@@ -2462,26 +2469,77 @@
       <c r="L70" s="5"/>
       <c r="M70" s="5"/>
       <c r="N70" s="5"/>
-      <c r="O70" s="9"/>
-      <c r="P70" s="9"/>
-      <c r="Q70" s="9"/>
-      <c r="R70" s="9"/>
-      <c r="S70" s="9"/>
-      <c r="T70" s="9"/>
-      <c r="U70" s="9"/>
-      <c r="V70" s="9"/>
+      <c r="O70" s="11"/>
+      <c r="P70" s="11"/>
+      <c r="Q70" s="11"/>
+      <c r="R70" s="11"/>
+      <c r="S70" s="11"/>
+      <c r="T70" s="11"/>
+      <c r="U70" s="11"/>
+      <c r="V70" s="11"/>
+    </row>
+    <row r="71" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A71" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C71" s="5"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="5"/>
+      <c r="H71" s="5"/>
+      <c r="I71" s="5"/>
+      <c r="J71" s="5"/>
+      <c r="K71" s="5"/>
+      <c r="L71" s="5"/>
+      <c r="M71" s="5"/>
+      <c r="N71" s="5"/>
+      <c r="O71" s="11"/>
+      <c r="P71" s="11"/>
+      <c r="Q71" s="11"/>
+      <c r="R71" s="11"/>
+      <c r="S71" s="11"/>
+      <c r="T71" s="11"/>
+      <c r="U71" s="11"/>
+      <c r="V71" s="11"/>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>46</v>
-      </c>
+      <c r="A72" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C72" s="5"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="5"/>
+      <c r="F72" s="5"/>
+      <c r="G72" s="5"/>
+      <c r="H72" s="5"/>
+      <c r="I72" s="5"/>
+      <c r="J72" s="5"/>
+      <c r="K72" s="5"/>
+      <c r="L72" s="5"/>
+      <c r="M72" s="5"/>
+      <c r="N72" s="5"/>
+      <c r="O72" s="11"/>
+      <c r="P72" s="11"/>
+      <c r="Q72" s="11"/>
+      <c r="R72" s="11"/>
+      <c r="S72" s="11"/>
+      <c r="T72" s="11"/>
+      <c r="U72" s="11"/>
+      <c r="V72" s="11"/>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C73" s="5"/>
       <c r="D73" s="5"/>
@@ -2495,21 +2553,21 @@
       <c r="L73" s="5"/>
       <c r="M73" s="5"/>
       <c r="N73" s="5"/>
-      <c r="O73" s="9"/>
-      <c r="P73" s="9"/>
-      <c r="Q73" s="9"/>
-      <c r="R73" s="9"/>
-      <c r="S73" s="9"/>
-      <c r="T73" s="9"/>
-      <c r="U73" s="9"/>
-      <c r="V73" s="9"/>
+      <c r="O73" s="11"/>
+      <c r="P73" s="11"/>
+      <c r="Q73" s="11"/>
+      <c r="R73" s="11"/>
+      <c r="S73" s="11"/>
+      <c r="T73" s="11"/>
+      <c r="U73" s="11"/>
+      <c r="V73" s="11"/>
     </row>
     <row r="74" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C74" s="5"/>
       <c r="D74" s="5"/>
@@ -2523,21 +2581,21 @@
       <c r="L74" s="5"/>
       <c r="M74" s="5"/>
       <c r="N74" s="5"/>
-      <c r="O74" s="9"/>
-      <c r="P74" s="9"/>
-      <c r="Q74" s="9"/>
-      <c r="R74" s="9"/>
-      <c r="S74" s="9"/>
-      <c r="T74" s="9"/>
-      <c r="U74" s="9"/>
-      <c r="V74" s="9"/>
+      <c r="O74" s="11"/>
+      <c r="P74" s="11"/>
+      <c r="Q74" s="11"/>
+      <c r="R74" s="11"/>
+      <c r="S74" s="11"/>
+      <c r="T74" s="11"/>
+      <c r="U74" s="11"/>
+      <c r="V74" s="11"/>
     </row>
     <row r="75" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C75" s="5"/>
       <c r="D75" s="5"/>
@@ -2551,21 +2609,21 @@
       <c r="L75" s="5"/>
       <c r="M75" s="5"/>
       <c r="N75" s="5"/>
-      <c r="O75" s="9"/>
-      <c r="P75" s="9"/>
-      <c r="Q75" s="9"/>
-      <c r="R75" s="9"/>
-      <c r="S75" s="9"/>
-      <c r="T75" s="9"/>
-      <c r="U75" s="9"/>
-      <c r="V75" s="9"/>
+      <c r="O75" s="11"/>
+      <c r="P75" s="11"/>
+      <c r="Q75" s="11"/>
+      <c r="R75" s="11"/>
+      <c r="S75" s="11"/>
+      <c r="T75" s="11"/>
+      <c r="U75" s="11"/>
+      <c r="V75" s="11"/>
     </row>
     <row r="76" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C76" s="5"/>
       <c r="D76" s="5"/>
@@ -2579,21 +2637,21 @@
       <c r="L76" s="5"/>
       <c r="M76" s="5"/>
       <c r="N76" s="5"/>
-      <c r="O76" s="9"/>
-      <c r="P76" s="9"/>
-      <c r="Q76" s="9"/>
-      <c r="R76" s="9"/>
-      <c r="S76" s="9"/>
-      <c r="T76" s="9"/>
-      <c r="U76" s="9"/>
-      <c r="V76" s="9"/>
+      <c r="O76" s="11"/>
+      <c r="P76" s="11"/>
+      <c r="Q76" s="11"/>
+      <c r="R76" s="11"/>
+      <c r="S76" s="11"/>
+      <c r="T76" s="11"/>
+      <c r="U76" s="11"/>
+      <c r="V76" s="11"/>
     </row>
     <row r="77" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C77" s="5"/>
       <c r="D77" s="5"/>
@@ -2607,21 +2665,21 @@
       <c r="L77" s="5"/>
       <c r="M77" s="5"/>
       <c r="N77" s="5"/>
-      <c r="O77" s="9"/>
-      <c r="P77" s="9"/>
-      <c r="Q77" s="9"/>
-      <c r="R77" s="9"/>
-      <c r="S77" s="9"/>
-      <c r="T77" s="9"/>
-      <c r="U77" s="9"/>
-      <c r="V77" s="9"/>
+      <c r="O77" s="11"/>
+      <c r="P77" s="11"/>
+      <c r="Q77" s="11"/>
+      <c r="R77" s="11"/>
+      <c r="S77" s="11"/>
+      <c r="T77" s="11"/>
+      <c r="U77" s="11"/>
+      <c r="V77" s="11"/>
     </row>
     <row r="78" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C78" s="5"/>
       <c r="D78" s="5"/>
@@ -2635,21 +2693,21 @@
       <c r="L78" s="5"/>
       <c r="M78" s="5"/>
       <c r="N78" s="5"/>
-      <c r="O78" s="9"/>
-      <c r="P78" s="9"/>
-      <c r="Q78" s="9"/>
-      <c r="R78" s="9"/>
-      <c r="S78" s="9"/>
-      <c r="T78" s="9"/>
-      <c r="U78" s="9"/>
-      <c r="V78" s="9"/>
+      <c r="O78" s="11"/>
+      <c r="P78" s="11"/>
+      <c r="Q78" s="11"/>
+      <c r="R78" s="11"/>
+      <c r="S78" s="11"/>
+      <c r="T78" s="11"/>
+      <c r="U78" s="11"/>
+      <c r="V78" s="11"/>
     </row>
     <row r="79" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C79" s="5"/>
       <c r="D79" s="5"/>
@@ -2663,74 +2721,23 @@
       <c r="L79" s="5"/>
       <c r="M79" s="5"/>
       <c r="N79" s="5"/>
-      <c r="O79" s="9"/>
-      <c r="P79" s="9"/>
-      <c r="Q79" s="9"/>
-      <c r="R79" s="9"/>
-      <c r="S79" s="9"/>
-      <c r="T79" s="9"/>
-      <c r="U79" s="9"/>
-      <c r="V79" s="9"/>
-    </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A80" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C80" s="5"/>
-      <c r="D80" s="5"/>
-      <c r="E80" s="5"/>
-      <c r="F80" s="5"/>
-      <c r="G80" s="5"/>
-      <c r="H80" s="5"/>
-      <c r="I80" s="5"/>
-      <c r="J80" s="5"/>
-      <c r="K80" s="5"/>
-      <c r="L80" s="5"/>
-      <c r="M80" s="5"/>
-      <c r="N80" s="5"/>
-      <c r="O80" s="9"/>
-      <c r="P80" s="9"/>
-      <c r="Q80" s="9"/>
-      <c r="R80" s="9"/>
-      <c r="S80" s="9"/>
-      <c r="T80" s="9"/>
-      <c r="U80" s="9"/>
-      <c r="V80" s="9"/>
+      <c r="O79" s="11"/>
+      <c r="P79" s="11"/>
+      <c r="Q79" s="11"/>
+      <c r="R79" s="11"/>
+      <c r="S79" s="11"/>
+      <c r="T79" s="11"/>
+      <c r="U79" s="11"/>
+      <c r="V79" s="11"/>
     </row>
     <row r="81" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A81" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C81" s="5"/>
-      <c r="D81" s="5"/>
-      <c r="E81" s="5"/>
-      <c r="F81" s="5"/>
-      <c r="G81" s="5"/>
-      <c r="H81" s="5"/>
-      <c r="I81" s="5"/>
-      <c r="J81" s="5"/>
-      <c r="K81" s="5"/>
-      <c r="L81" s="5"/>
-      <c r="M81" s="5"/>
-      <c r="N81" s="5"/>
-      <c r="O81" s="9"/>
-      <c r="P81" s="9"/>
-      <c r="Q81" s="9"/>
-      <c r="R81" s="9"/>
-      <c r="S81" s="9"/>
-      <c r="T81" s="9"/>
-      <c r="U81" s="9"/>
-      <c r="V81" s="9"/>
+      <c r="A81" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="82" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>5</v>
@@ -2747,18 +2754,18 @@
       <c r="L82" s="5"/>
       <c r="M82" s="5"/>
       <c r="N82" s="5"/>
-      <c r="O82" s="9"/>
-      <c r="P82" s="9"/>
-      <c r="Q82" s="9"/>
-      <c r="R82" s="9"/>
-      <c r="S82" s="9"/>
-      <c r="T82" s="9"/>
-      <c r="U82" s="9"/>
-      <c r="V82" s="9"/>
+      <c r="O82" s="11"/>
+      <c r="P82" s="11"/>
+      <c r="Q82" s="11"/>
+      <c r="R82" s="11"/>
+      <c r="S82" s="11"/>
+      <c r="T82" s="11"/>
+      <c r="U82" s="11"/>
+      <c r="V82" s="11"/>
     </row>
     <row r="83" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>5</v>
@@ -2775,18 +2782,18 @@
       <c r="L83" s="5"/>
       <c r="M83" s="5"/>
       <c r="N83" s="5"/>
-      <c r="O83" s="9"/>
-      <c r="P83" s="9"/>
-      <c r="Q83" s="9"/>
-      <c r="R83" s="9"/>
-      <c r="S83" s="9"/>
-      <c r="T83" s="9"/>
-      <c r="U83" s="9"/>
-      <c r="V83" s="9"/>
+      <c r="O83" s="11"/>
+      <c r="P83" s="11"/>
+      <c r="Q83" s="11"/>
+      <c r="R83" s="11"/>
+      <c r="S83" s="11"/>
+      <c r="T83" s="11"/>
+      <c r="U83" s="11"/>
+      <c r="V83" s="11"/>
     </row>
     <row r="84" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>5</v>
@@ -2803,18 +2810,18 @@
       <c r="L84" s="5"/>
       <c r="M84" s="5"/>
       <c r="N84" s="5"/>
-      <c r="O84" s="9"/>
-      <c r="P84" s="9"/>
-      <c r="Q84" s="9"/>
-      <c r="R84" s="9"/>
-      <c r="S84" s="9"/>
-      <c r="T84" s="9"/>
-      <c r="U84" s="9"/>
-      <c r="V84" s="9"/>
+      <c r="O84" s="11"/>
+      <c r="P84" s="11"/>
+      <c r="Q84" s="11"/>
+      <c r="R84" s="11"/>
+      <c r="S84" s="11"/>
+      <c r="T84" s="11"/>
+      <c r="U84" s="11"/>
+      <c r="V84" s="11"/>
     </row>
     <row r="85" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>5</v>
@@ -2831,18 +2838,18 @@
       <c r="L85" s="5"/>
       <c r="M85" s="5"/>
       <c r="N85" s="5"/>
-      <c r="O85" s="9"/>
-      <c r="P85" s="9"/>
-      <c r="Q85" s="9"/>
-      <c r="R85" s="9"/>
-      <c r="S85" s="9"/>
-      <c r="T85" s="9"/>
-      <c r="U85" s="9"/>
-      <c r="V85" s="9"/>
+      <c r="O85" s="11"/>
+      <c r="P85" s="11"/>
+      <c r="Q85" s="11"/>
+      <c r="R85" s="11"/>
+      <c r="S85" s="11"/>
+      <c r="T85" s="11"/>
+      <c r="U85" s="11"/>
+      <c r="V85" s="11"/>
     </row>
     <row r="86" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>5</v>
@@ -2859,14 +2866,266 @@
       <c r="L86" s="5"/>
       <c r="M86" s="5"/>
       <c r="N86" s="5"/>
-      <c r="O86" s="9"/>
-      <c r="P86" s="9"/>
-      <c r="Q86" s="9"/>
-      <c r="R86" s="9"/>
-      <c r="S86" s="9"/>
-      <c r="T86" s="9"/>
-      <c r="U86" s="9"/>
-      <c r="V86" s="9"/>
+      <c r="O86" s="11"/>
+      <c r="P86" s="11"/>
+      <c r="Q86" s="11"/>
+      <c r="R86" s="11"/>
+      <c r="S86" s="11"/>
+      <c r="T86" s="11"/>
+      <c r="U86" s="11"/>
+      <c r="V86" s="11"/>
+    </row>
+    <row r="87" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A87" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C87" s="5"/>
+      <c r="D87" s="5"/>
+      <c r="E87" s="5"/>
+      <c r="F87" s="5"/>
+      <c r="G87" s="5"/>
+      <c r="H87" s="5"/>
+      <c r="I87" s="5"/>
+      <c r="J87" s="5"/>
+      <c r="K87" s="5"/>
+      <c r="L87" s="5"/>
+      <c r="M87" s="5"/>
+      <c r="N87" s="5"/>
+      <c r="O87" s="11"/>
+      <c r="P87" s="11"/>
+      <c r="Q87" s="11"/>
+      <c r="R87" s="11"/>
+      <c r="S87" s="11"/>
+      <c r="T87" s="11"/>
+      <c r="U87" s="11"/>
+      <c r="V87" s="11"/>
+    </row>
+    <row r="88" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A88" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C88" s="5"/>
+      <c r="D88" s="5"/>
+      <c r="E88" s="5"/>
+      <c r="F88" s="5"/>
+      <c r="G88" s="5"/>
+      <c r="H88" s="5"/>
+      <c r="I88" s="5"/>
+      <c r="J88" s="5"/>
+      <c r="K88" s="5"/>
+      <c r="L88" s="5"/>
+      <c r="M88" s="5"/>
+      <c r="N88" s="5"/>
+      <c r="O88" s="11"/>
+      <c r="P88" s="11"/>
+      <c r="Q88" s="11"/>
+      <c r="R88" s="11"/>
+      <c r="S88" s="11"/>
+      <c r="T88" s="11"/>
+      <c r="U88" s="11"/>
+      <c r="V88" s="11"/>
+    </row>
+    <row r="89" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A89" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C89" s="5"/>
+      <c r="D89" s="5"/>
+      <c r="E89" s="5"/>
+      <c r="F89" s="5"/>
+      <c r="G89" s="5"/>
+      <c r="H89" s="5"/>
+      <c r="I89" s="5"/>
+      <c r="J89" s="5"/>
+      <c r="K89" s="5"/>
+      <c r="L89" s="5"/>
+      <c r="M89" s="5"/>
+      <c r="N89" s="5"/>
+      <c r="O89" s="11"/>
+      <c r="P89" s="11"/>
+      <c r="Q89" s="11"/>
+      <c r="R89" s="11"/>
+      <c r="S89" s="11"/>
+      <c r="T89" s="11"/>
+      <c r="U89" s="11"/>
+      <c r="V89" s="11"/>
+    </row>
+    <row r="90" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A90" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C90" s="5"/>
+      <c r="D90" s="5"/>
+      <c r="E90" s="5"/>
+      <c r="F90" s="5"/>
+      <c r="G90" s="5"/>
+      <c r="H90" s="5"/>
+      <c r="I90" s="5"/>
+      <c r="J90" s="5"/>
+      <c r="K90" s="5"/>
+      <c r="L90" s="5"/>
+      <c r="M90" s="5"/>
+      <c r="N90" s="5"/>
+      <c r="O90" s="11"/>
+      <c r="P90" s="11"/>
+      <c r="Q90" s="11"/>
+      <c r="R90" s="11"/>
+      <c r="S90" s="11"/>
+      <c r="T90" s="11"/>
+      <c r="U90" s="11"/>
+      <c r="V90" s="11"/>
+    </row>
+    <row r="91" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A91" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C91" s="5"/>
+      <c r="D91" s="5"/>
+      <c r="E91" s="5"/>
+      <c r="F91" s="5"/>
+      <c r="G91" s="5"/>
+      <c r="H91" s="5"/>
+      <c r="I91" s="5"/>
+      <c r="J91" s="5"/>
+      <c r="K91" s="5"/>
+      <c r="L91" s="5"/>
+      <c r="M91" s="5"/>
+      <c r="N91" s="5"/>
+      <c r="O91" s="11"/>
+      <c r="P91" s="11"/>
+      <c r="Q91" s="11"/>
+      <c r="R91" s="11"/>
+      <c r="S91" s="11"/>
+      <c r="T91" s="11"/>
+      <c r="U91" s="11"/>
+      <c r="V91" s="11"/>
+    </row>
+    <row r="92" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A92" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C92" s="5"/>
+      <c r="D92" s="5"/>
+      <c r="E92" s="5"/>
+      <c r="F92" s="5"/>
+      <c r="G92" s="5"/>
+      <c r="H92" s="5"/>
+      <c r="I92" s="5"/>
+      <c r="J92" s="5"/>
+      <c r="K92" s="5"/>
+      <c r="L92" s="5"/>
+      <c r="M92" s="5"/>
+      <c r="N92" s="5"/>
+      <c r="O92" s="11"/>
+      <c r="P92" s="11"/>
+      <c r="Q92" s="11"/>
+      <c r="R92" s="11"/>
+      <c r="S92" s="11"/>
+      <c r="T92" s="11"/>
+      <c r="U92" s="11"/>
+      <c r="V92" s="11"/>
+    </row>
+    <row r="93" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A93" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C93" s="5"/>
+      <c r="D93" s="5"/>
+      <c r="E93" s="5"/>
+      <c r="F93" s="5"/>
+      <c r="G93" s="5"/>
+      <c r="H93" s="5"/>
+      <c r="I93" s="5"/>
+      <c r="J93" s="5"/>
+      <c r="K93" s="5"/>
+      <c r="L93" s="5"/>
+      <c r="M93" s="5"/>
+      <c r="N93" s="5"/>
+      <c r="O93" s="11"/>
+      <c r="P93" s="11"/>
+      <c r="Q93" s="11"/>
+      <c r="R93" s="11"/>
+      <c r="S93" s="11"/>
+      <c r="T93" s="11"/>
+      <c r="U93" s="11"/>
+      <c r="V93" s="11"/>
+    </row>
+    <row r="94" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A94" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C94" s="5"/>
+      <c r="D94" s="5"/>
+      <c r="E94" s="5"/>
+      <c r="F94" s="5"/>
+      <c r="G94" s="5"/>
+      <c r="H94" s="5"/>
+      <c r="I94" s="5"/>
+      <c r="J94" s="5"/>
+      <c r="K94" s="5"/>
+      <c r="L94" s="5"/>
+      <c r="M94" s="5"/>
+      <c r="N94" s="5"/>
+      <c r="O94" s="11"/>
+      <c r="P94" s="11"/>
+      <c r="Q94" s="11"/>
+      <c r="R94" s="11"/>
+      <c r="S94" s="11"/>
+      <c r="T94" s="11"/>
+      <c r="U94" s="11"/>
+      <c r="V94" s="11"/>
+    </row>
+    <row r="95" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A95" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C95" s="5"/>
+      <c r="D95" s="5"/>
+      <c r="E95" s="5"/>
+      <c r="F95" s="5"/>
+      <c r="G95" s="5"/>
+      <c r="H95" s="5"/>
+      <c r="I95" s="5"/>
+      <c r="J95" s="5"/>
+      <c r="K95" s="5"/>
+      <c r="L95" s="5"/>
+      <c r="M95" s="5"/>
+      <c r="N95" s="5"/>
+      <c r="O95" s="11"/>
+      <c r="P95" s="11"/>
+      <c r="Q95" s="11"/>
+      <c r="R95" s="11"/>
+      <c r="S95" s="11"/>
+      <c r="T95" s="11"/>
+      <c r="U95" s="11"/>
+      <c r="V95" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>